<commit_message>
Updated leaderboard for r2
</commit_message>
<xml_diff>
--- a/public/res/leaderboards/Advanced.xlsx
+++ b/public/res/leaderboards/Advanced.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lawrence\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lawrence\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DABC261-3C12-408C-807E-A0AFCA82090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2D808C5-D424-4055-9FBC-DF0D7C436005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{231F0BEC-F623-41AC-8721-73F4116A0546}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t>#</t>
   </si>
@@ -185,10 +185,91 @@
     <t>Austin Yam</t>
   </si>
   <si>
-    <t>Itsuki Cheng</t>
-  </si>
-  <si>
     <t>Jun Chen</t>
+  </si>
+  <si>
+    <t>Zichuan Zou</t>
+  </si>
+  <si>
+    <t>Kaan Yilmaz</t>
+  </si>
+  <si>
+    <t>Keyur Gohel</t>
+  </si>
+  <si>
+    <t>finnegan clapp</t>
+  </si>
+  <si>
+    <t>Rudhra Khandelwal</t>
+  </si>
+  <si>
+    <t>avicknash dayanandan</t>
+  </si>
+  <si>
+    <t>Ty Gredina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyrus Han </t>
+  </si>
+  <si>
+    <t>Ziggy Guan</t>
+  </si>
+  <si>
+    <t>scott zhou</t>
+  </si>
+  <si>
+    <t>Andrew Nguyen</t>
+  </si>
+  <si>
+    <t>Izac Jie Ming Ooi</t>
+  </si>
+  <si>
+    <t>Jackie Xie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jordan Rao </t>
+  </si>
+  <si>
+    <t>Jason You</t>
+  </si>
+  <si>
+    <t>Kevin Mogil</t>
+  </si>
+  <si>
+    <t>Tanvir Singh</t>
+  </si>
+  <si>
+    <t>Corey Gendala</t>
+  </si>
+  <si>
+    <t>Aashay Deo</t>
+  </si>
+  <si>
+    <t>Santiago Sassman</t>
+  </si>
+  <si>
+    <t>avnish ranchigoda</t>
+  </si>
+  <si>
+    <t>Zichen Xue</t>
+  </si>
+  <si>
+    <t>Vojtech Zeman</t>
+  </si>
+  <si>
+    <t>Zabrain Haider</t>
+  </si>
+  <si>
+    <t>Cas Chng</t>
+  </si>
+  <si>
+    <t>yi tang</t>
+  </si>
+  <si>
+    <t>kalabe araya</t>
+  </si>
+  <si>
+    <t>kevin gonzalez arias</t>
   </si>
 </sst>
 </file>
@@ -589,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A97B47B5-A6D7-41E5-A619-C36FE2241088}">
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -626,13 +707,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C2">
-        <v>146300</v>
+        <v>71000</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>213600</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -647,7 +728,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>146300</v>
+        <v>284600</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -655,13 +736,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3">
-        <v>120000</v>
+        <v>118600</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>123300</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -676,7 +757,7 @@
         <v>0</v>
       </c>
       <c r="I3">
-        <v>120000</v>
+        <v>241900</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -684,13 +765,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="C4">
-        <v>118600</v>
+        <v>54100</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>139300</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -705,7 +786,7 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>118600</v>
+        <v>178400</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -713,13 +794,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="C5">
-        <v>118000</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>150700</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -734,7 +815,7 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>118000</v>
+        <v>150700</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -742,10 +823,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C6">
-        <v>111300</v>
+        <v>146300</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -763,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>111300</v>
+        <v>131300</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -771,13 +852,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="C7">
-        <v>71900</v>
+        <v>45900</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>80700</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -792,7 +873,7 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>71900</v>
+        <v>126600</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
@@ -800,13 +881,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C8">
-        <v>71100</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>124800</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -821,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>71100</v>
+        <v>124800</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -829,10 +910,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C9">
-        <v>71000</v>
+        <v>120000</v>
       </c>
       <c r="D9">
         <v>0</v>
@@ -850,7 +931,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>71000</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
@@ -858,10 +939,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C10">
-        <v>65800</v>
+        <v>118000</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -879,7 +960,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>65800</v>
+        <v>118000</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
@@ -887,13 +968,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C11">
-        <v>65600</v>
+        <v>35500</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>79200</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -908,7 +989,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>65600</v>
+        <v>114700</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
@@ -916,10 +997,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C12">
-        <v>59800</v>
+        <v>111300</v>
       </c>
       <c r="D12">
         <v>0</v>
@@ -937,7 +1018,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>59800</v>
+        <v>111300</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
@@ -945,13 +1026,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C13">
-        <v>58600</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>94500</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -966,7 +1047,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>58600</v>
+        <v>94500</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
@@ -974,13 +1055,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14">
-        <v>56200</v>
+        <v>59800</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>31200</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -995,7 +1076,7 @@
         <v>0</v>
       </c>
       <c r="I14">
-        <v>56200</v>
+        <v>91000</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
@@ -1003,13 +1084,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="C15">
-        <v>55500</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>88200</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -1024,7 +1105,7 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>55500</v>
+        <v>88200</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
@@ -1032,13 +1113,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="C16">
-        <v>54600</v>
+        <v>0</v>
       </c>
       <c r="D16">
-        <v>0</v>
+        <v>84400</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -1053,7 +1134,7 @@
         <v>0</v>
       </c>
       <c r="I16">
-        <v>54600</v>
+        <v>84400</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
@@ -1061,13 +1142,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C17">
-        <v>54100</v>
+        <v>56200</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>11400</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -1082,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="I17">
-        <v>54100</v>
+        <v>67600</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
@@ -1090,13 +1171,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="C18">
-        <v>51000</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <v>66400</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1111,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>51000</v>
+        <v>66400</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
@@ -1119,13 +1200,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C19">
-        <v>50400</v>
+        <v>11400</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <v>55000</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -1140,7 +1221,7 @@
         <v>0</v>
       </c>
       <c r="I19">
-        <v>50400</v>
+        <v>66400</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
@@ -1148,10 +1229,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C20">
-        <v>46200</v>
+        <v>65800</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1169,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="I20">
-        <v>46200</v>
+        <v>65800</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
@@ -1177,10 +1258,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C21">
-        <v>45900</v>
+        <v>65600</v>
       </c>
       <c r="D21">
         <v>0</v>
@@ -1198,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="I21">
-        <v>45900</v>
+        <v>65600</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
@@ -1206,13 +1287,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="C22">
-        <v>45500</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>60900</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -1227,7 +1308,7 @@
         <v>0</v>
       </c>
       <c r="I22">
-        <v>45500</v>
+        <v>60900</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
@@ -1235,10 +1316,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C23">
-        <v>39400</v>
+        <v>58600</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1256,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="I23">
-        <v>39400</v>
+        <v>58600</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
@@ -1264,13 +1345,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
       <c r="C24">
-        <v>37700</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>58500</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -1285,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="I24">
-        <v>37700</v>
+        <v>58500</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
@@ -1293,10 +1374,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C25">
-        <v>35500</v>
+        <v>71900</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -1314,7 +1395,7 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <v>35500</v>
+        <v>56900</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
@@ -1322,10 +1403,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C26">
-        <v>35400</v>
+        <v>71100</v>
       </c>
       <c r="D26">
         <v>0</v>
@@ -1343,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="I26">
-        <v>35400</v>
+        <v>56100</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
@@ -1351,10 +1432,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="C27">
-        <v>34900</v>
+        <v>55500</v>
       </c>
       <c r="D27">
         <v>0</v>
@@ -1372,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="I27">
-        <v>34900</v>
+        <v>55500</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
@@ -1380,13 +1461,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="C28">
-        <v>32100</v>
+        <v>0</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>53300</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -1401,7 +1482,7 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>32100</v>
+        <v>53300</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
@@ -1409,13 +1490,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C29">
-        <v>31200</v>
+        <v>0</v>
       </c>
       <c r="D29">
-        <v>0</v>
+        <v>52000</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1430,7 +1511,7 @@
         <v>0</v>
       </c>
       <c r="I29">
-        <v>31200</v>
+        <v>52000</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
@@ -1438,10 +1519,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="C30">
-        <v>30000</v>
+        <v>51000</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -1459,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="I30">
-        <v>30000</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
@@ -1467,10 +1548,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C31">
-        <v>29400</v>
+        <v>50400</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -1488,7 +1569,7 @@
         <v>0</v>
       </c>
       <c r="I31">
-        <v>29400</v>
+        <v>50400</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
@@ -1496,13 +1577,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="C32">
-        <v>29200</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>49800</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -1517,7 +1598,7 @@
         <v>0</v>
       </c>
       <c r="I32">
-        <v>29200</v>
+        <v>49800</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
@@ -1525,13 +1606,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="C33">
-        <v>27300</v>
+        <v>0</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>49700</v>
       </c>
       <c r="E33">
         <v>0</v>
@@ -1546,7 +1627,7 @@
         <v>0</v>
       </c>
       <c r="I33">
-        <v>27300</v>
+        <v>49700</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
@@ -1554,10 +1635,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="C34">
-        <v>27200</v>
+        <v>46200</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -1575,7 +1656,7 @@
         <v>0</v>
       </c>
       <c r="I34">
-        <v>27200</v>
+        <v>46200</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
@@ -1583,10 +1664,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="C35">
-        <v>25500</v>
+        <v>45900</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -1604,7 +1685,7 @@
         <v>0</v>
       </c>
       <c r="I35">
-        <v>25500</v>
+        <v>45900</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
@@ -1612,10 +1693,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="C36">
-        <v>25400</v>
+        <v>45500</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -1633,7 +1714,7 @@
         <v>0</v>
       </c>
       <c r="I36">
-        <v>25400</v>
+        <v>45500</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
@@ -1641,13 +1722,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C37">
-        <v>21600</v>
+        <v>0</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>43700</v>
       </c>
       <c r="E37">
         <v>0</v>
@@ -1662,7 +1743,7 @@
         <v>0</v>
       </c>
       <c r="I37">
-        <v>21600</v>
+        <v>43700</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
@@ -1670,13 +1751,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="C38">
-        <v>18800</v>
+        <v>0</v>
       </c>
       <c r="D38">
-        <v>0</v>
+        <v>43500</v>
       </c>
       <c r="E38">
         <v>0</v>
@@ -1691,7 +1772,7 @@
         <v>0</v>
       </c>
       <c r="I38">
-        <v>18800</v>
+        <v>43500</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
@@ -1699,10 +1780,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C39">
-        <v>16800</v>
+        <v>54600</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -1720,7 +1801,7 @@
         <v>0</v>
       </c>
       <c r="I39">
-        <v>16800</v>
+        <v>39600</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
@@ -1728,10 +1809,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="C40">
-        <v>13100</v>
+        <v>39400</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -1749,7 +1830,7 @@
         <v>0</v>
       </c>
       <c r="I40">
-        <v>13100</v>
+        <v>39400</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
@@ -1757,13 +1838,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="C41">
-        <v>12400</v>
+        <v>0</v>
       </c>
       <c r="D41">
-        <v>0</v>
+        <v>39400</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -1778,7 +1859,7 @@
         <v>0</v>
       </c>
       <c r="I41">
-        <v>12400</v>
+        <v>39400</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
@@ -1786,28 +1867,811 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>39000</v>
+      </c>
+      <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>0</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
+      </c>
+      <c r="I42">
+        <v>39000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>67</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>37500</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43">
+        <v>0</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>37500</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>34</v>
+      </c>
+      <c r="C44">
+        <v>34900</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>0</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>34900</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>68</v>
+      </c>
+      <c r="C45">
+        <v>34400</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
+      </c>
+      <c r="I45">
+        <v>34400</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46">
+        <v>27300</v>
+      </c>
+      <c r="D46">
+        <v>20500</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>0</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
+      </c>
+      <c r="I46">
+        <v>32800</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>35</v>
+      </c>
+      <c r="C47">
+        <v>32100</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47">
+        <v>0</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
+      </c>
+      <c r="I47">
+        <v>32100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>69</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>31600</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>0</v>
+      </c>
+      <c r="G48">
+        <v>0</v>
+      </c>
+      <c r="H48">
+        <v>0</v>
+      </c>
+      <c r="I48">
+        <v>31600</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>70</v>
+      </c>
+      <c r="C49">
+        <v>31500</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49">
+        <v>0</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>31500</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50">
         <v>49</v>
       </c>
-      <c r="C42">
+      <c r="B50" t="s">
+        <v>36</v>
+      </c>
+      <c r="C50">
+        <v>31200</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>0</v>
+      </c>
+      <c r="G50">
+        <v>0</v>
+      </c>
+      <c r="H50">
+        <v>0</v>
+      </c>
+      <c r="I50">
+        <v>31200</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>37</v>
+      </c>
+      <c r="C51">
+        <v>30000</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>0</v>
+      </c>
+      <c r="F51">
+        <v>0</v>
+      </c>
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>42</v>
+      </c>
+      <c r="C52">
+        <v>25500</v>
+      </c>
+      <c r="D52">
+        <v>19400</v>
+      </c>
+      <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52">
+        <v>0</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52">
+        <v>29900</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>38</v>
+      </c>
+      <c r="C53">
+        <v>29400</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53">
+        <v>0</v>
+      </c>
+      <c r="F53">
+        <v>0</v>
+      </c>
+      <c r="G53">
+        <v>0</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53">
+        <v>29400</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>41</v>
+      </c>
+      <c r="C54">
+        <v>27200</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54">
+        <v>0</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>27200</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>43</v>
+      </c>
+      <c r="C55">
+        <v>25400</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>0</v>
+      </c>
+      <c r="G55">
+        <v>0</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55">
+        <v>25400</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>71</v>
+      </c>
+      <c r="C56">
+        <v>24000</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>31</v>
+      </c>
+      <c r="C57">
+        <v>37700</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>0</v>
+      </c>
+      <c r="G57">
+        <v>0</v>
+      </c>
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57">
+        <v>22700</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <v>22600</v>
+      </c>
+      <c r="E58">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>0</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>22600</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>44</v>
+      </c>
+      <c r="C59">
+        <v>21600</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>0</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
+        <v>21600</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>33</v>
+      </c>
+      <c r="C60">
+        <v>35400</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>0</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60">
+        <v>20400</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>73</v>
+      </c>
+      <c r="C61">
+        <v>33200</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>0</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61">
+        <v>18200</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>46</v>
+      </c>
+      <c r="C62">
+        <v>16800</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>0</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62">
+        <v>16800</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>15600</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>0</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>15600</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>39</v>
+      </c>
+      <c r="C64">
+        <v>29200</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>0</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>14200</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>47</v>
+      </c>
+      <c r="C65">
+        <v>13100</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>0</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>13100</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>48</v>
+      </c>
+      <c r="C66">
         <v>8700</v>
       </c>
-      <c r="D42">
-        <v>0</v>
-      </c>
-      <c r="E42">
-        <v>0</v>
-      </c>
-      <c r="F42">
-        <v>0</v>
-      </c>
-      <c r="G42">
-        <v>0</v>
-      </c>
-      <c r="H42">
-        <v>0</v>
-      </c>
-      <c r="I42">
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>0</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66">
         <v>8700</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>75</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>3900</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>45</v>
+      </c>
+      <c r="C68">
+        <v>18800</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68">
+        <v>3800</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>76</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>3300</v>
+      </c>
+      <c r="E69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <v>0</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69">
+        <v>3300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>